<commit_message>
FIX: Fixes from copilot and refactor a bunch of code
(sorry!)
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/SEQUENCE.xlsx
+++ b/xlsx/tests/calc_tests/SEQUENCE.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6429092-828B-F541-9297-945E9E3D45EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962B2A32-B52E-CA4B-8D1E-3FF4C075AE27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="620" windowWidth="16820" windowHeight="18560" xr2:uid="{D28D3A38-53E7-8E4B-8D0A-473C04C3AFED}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="16820" windowHeight="18560" xr2:uid="{D28D3A38-53E7-8E4B-8D0A-473C04C3AFED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -500,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7F16674-7FCE-844C-B851-4088E514E246}">
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
@@ -691,12 +691,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="G17">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C18" t="e" cm="1">
         <f t="array" ref="C18">_xlfn.SEQUENCE(-1)</f>
         <v>#VALUE!</v>
@@ -709,14 +709,67 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="G19">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="G20">
         <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A23" cm="1">
+        <f t="array" ref="A23:A25">_xlfn.SEQUENCE(3,,10)</f>
+        <v>10</v>
+      </c>
+      <c r="C23" cm="1">
+        <f t="array" ref="C23:N23">_xlfn.SEQUENCE(,12,,2.5)</f>
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>3.5</v>
+      </c>
+      <c r="E23">
+        <v>6</v>
+      </c>
+      <c r="F23">
+        <v>8.5</v>
+      </c>
+      <c r="G23">
+        <v>11</v>
+      </c>
+      <c r="H23">
+        <v>13.5</v>
+      </c>
+      <c r="I23">
+        <v>16</v>
+      </c>
+      <c r="J23">
+        <v>18.5</v>
+      </c>
+      <c r="K23">
+        <v>21</v>
+      </c>
+      <c r="L23">
+        <v>23.5</v>
+      </c>
+      <c r="M23">
+        <v>26</v>
+      </c>
+      <c r="N23">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>